<commit_message>
was missing WWARN pd data - whoops
</commit_message>
<xml_diff>
--- a/analysis/data-raw/PMID_pd_replace.xlsx
+++ b/analysis/data-raw/PMID_pd_replace.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rverity/Dropbox/Bob/Work/My Programs/Mapping/scrub/analysis/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08DFB096-66E7-5F44-87A1-A664E4C883BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025D262E-31F7-B742-BD04-FAD2862EF6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="1560" windowWidth="23500" windowHeight="16760" firstSheet="32" activeTab="40" xr2:uid="{DA1909FE-6D53-CC42-B275-AE2BCB499241}"/>
+    <workbookView xWindow="1180" yWindow="5220" windowWidth="23500" windowHeight="16760" firstSheet="7" activeTab="10" xr2:uid="{DA1909FE-6D53-CC42-B275-AE2BCB499241}"/>
   </bookViews>
   <sheets>
     <sheet name="11926004" sheetId="2" r:id="rId1"/>
@@ -2545,7 +2545,7 @@
         <v>2015</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -30252,7 +30252,7 @@
         <v>2012</v>
       </c>
       <c r="I4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J4">
         <v>5</v>

</xml_diff>